<commit_message>
Correction to aircraft estimates, part 1 of calbrated variables
</commit_message>
<xml_diff>
--- a/InputData/bldgs/RBFF/Recipient Buildings Fuel Fractions.xlsx
+++ b/InputData/bldgs/RBFF/Recipient Buildings Fuel Fractions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23901"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olivia\Documents\EPS_Models by Region\United States\NEW_US\InputData\bldgs\RBFF\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary Francis Swint\Vensim\eps-indonesia\InputData\bldgs\RBFF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE4E3257-D795-4A92-804F-0180AA3862CC}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2972CEC-1BBB-4C39-9A9E-59E8CB42AE31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9660" yWindow="1080" windowWidth="17205" windowHeight="16065" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="960" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -135,10 +135,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -458,17 +457,17 @@
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+      <c r="A7" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="A8" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+      <c r="A9" t="s">
         <v>5</v>
       </c>
     </row>
@@ -502,42 +501,42 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.28515625" customWidth="1"/>
-    <col min="2" max="6" width="17.28515625" style="5" customWidth="1"/>
+    <col min="2" max="6" width="17.28515625" style="4" customWidth="1"/>
     <col min="7" max="11" width="17.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:11" s="5" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="3" t="s">
         <v>20</v>
       </c>
     </row>
@@ -545,34 +544,34 @@
       <c r="A2" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="5">
-        <v>1</v>
-      </c>
-      <c r="C2" s="5">
-        <v>1</v>
-      </c>
-      <c r="D2" s="5">
-        <v>1</v>
-      </c>
-      <c r="E2" s="5">
-        <v>1</v>
-      </c>
-      <c r="F2" s="5">
-        <v>1</v>
-      </c>
-      <c r="G2" s="5">
-        <v>0</v>
-      </c>
-      <c r="H2" s="5">
-        <v>1</v>
-      </c>
-      <c r="I2" s="5">
-        <v>1</v>
-      </c>
-      <c r="J2" s="5">
-        <v>1</v>
-      </c>
-      <c r="K2" s="5">
+      <c r="B2" s="4">
+        <v>1</v>
+      </c>
+      <c r="C2" s="4">
+        <v>1</v>
+      </c>
+      <c r="D2" s="4">
+        <v>1</v>
+      </c>
+      <c r="E2" s="4">
+        <v>1</v>
+      </c>
+      <c r="F2" s="4">
+        <v>0</v>
+      </c>
+      <c r="G2" s="4">
+        <v>0</v>
+      </c>
+      <c r="H2" s="4">
+        <v>1</v>
+      </c>
+      <c r="I2" s="4">
+        <v>1</v>
+      </c>
+      <c r="J2" s="4">
+        <v>1</v>
+      </c>
+      <c r="K2" s="4">
         <v>1</v>
       </c>
     </row>
@@ -580,34 +579,34 @@
       <c r="A3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="5">
-        <v>0</v>
-      </c>
-      <c r="C3" s="5">
-        <v>0</v>
-      </c>
-      <c r="D3" s="5">
-        <v>0</v>
-      </c>
-      <c r="E3" s="5">
-        <v>0</v>
-      </c>
-      <c r="F3" s="5">
-        <v>0</v>
-      </c>
-      <c r="G3" s="5">
-        <v>0</v>
-      </c>
-      <c r="H3" s="5">
-        <v>0</v>
-      </c>
-      <c r="I3" s="5">
-        <v>0</v>
-      </c>
-      <c r="J3" s="5">
-        <v>0</v>
-      </c>
-      <c r="K3" s="5">
+      <c r="B3" s="4">
+        <v>0</v>
+      </c>
+      <c r="C3" s="4">
+        <v>0</v>
+      </c>
+      <c r="D3" s="4">
+        <v>0</v>
+      </c>
+      <c r="E3" s="4">
+        <v>0</v>
+      </c>
+      <c r="F3" s="4">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4">
+        <v>0</v>
+      </c>
+      <c r="I3" s="4">
+        <v>0</v>
+      </c>
+      <c r="J3" s="4">
+        <v>0</v>
+      </c>
+      <c r="K3" s="4">
         <v>0</v>
       </c>
     </row>
@@ -615,34 +614,34 @@
       <c r="A4" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="5">
-        <v>0</v>
-      </c>
-      <c r="C4" s="5">
-        <v>0</v>
-      </c>
-      <c r="D4" s="5">
-        <v>0</v>
-      </c>
-      <c r="E4" s="5">
-        <v>0</v>
-      </c>
-      <c r="F4" s="5">
-        <v>0</v>
-      </c>
-      <c r="G4" s="5">
-        <v>0</v>
-      </c>
-      <c r="H4" s="5">
-        <v>0</v>
-      </c>
-      <c r="I4" s="5">
-        <v>0</v>
-      </c>
-      <c r="J4" s="5">
-        <v>0</v>
-      </c>
-      <c r="K4" s="5">
+      <c r="B4" s="4">
+        <v>0</v>
+      </c>
+      <c r="C4" s="4">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4">
+        <v>0</v>
+      </c>
+      <c r="E4" s="4">
+        <v>0</v>
+      </c>
+      <c r="F4" s="4">
+        <v>0</v>
+      </c>
+      <c r="G4" s="4">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4">
+        <v>0</v>
+      </c>
+      <c r="I4" s="4">
+        <v>0</v>
+      </c>
+      <c r="J4" s="4">
+        <v>0</v>
+      </c>
+      <c r="K4" s="4">
         <v>0</v>
       </c>
     </row>
@@ -650,34 +649,34 @@
       <c r="A5" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="5">
-        <v>0</v>
-      </c>
-      <c r="C5" s="5">
-        <v>0</v>
-      </c>
-      <c r="D5" s="5">
-        <v>0</v>
-      </c>
-      <c r="E5" s="5">
-        <v>0</v>
-      </c>
-      <c r="F5" s="5">
-        <v>0</v>
-      </c>
-      <c r="G5" s="5">
-        <v>0</v>
-      </c>
-      <c r="H5" s="5">
-        <v>0</v>
-      </c>
-      <c r="I5" s="5">
-        <v>0</v>
-      </c>
-      <c r="J5" s="5">
-        <v>0</v>
-      </c>
-      <c r="K5" s="5">
+      <c r="B5" s="4">
+        <v>0</v>
+      </c>
+      <c r="C5" s="4">
+        <v>0</v>
+      </c>
+      <c r="D5" s="4">
+        <v>0</v>
+      </c>
+      <c r="E5" s="4">
+        <v>0</v>
+      </c>
+      <c r="F5" s="4">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4">
+        <v>0</v>
+      </c>
+      <c r="H5" s="4">
+        <v>0</v>
+      </c>
+      <c r="I5" s="4">
+        <v>0</v>
+      </c>
+      <c r="J5" s="4">
+        <v>0</v>
+      </c>
+      <c r="K5" s="4">
         <v>0</v>
       </c>
     </row>
@@ -685,34 +684,34 @@
       <c r="A6" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="5">
-        <v>0</v>
-      </c>
-      <c r="C6" s="5">
-        <v>0</v>
-      </c>
-      <c r="D6" s="5">
-        <v>0</v>
-      </c>
-      <c r="E6" s="5">
-        <v>0</v>
-      </c>
-      <c r="F6" s="5">
-        <v>0</v>
-      </c>
-      <c r="G6" s="5">
-        <v>0</v>
-      </c>
-      <c r="H6" s="5">
-        <v>0</v>
-      </c>
-      <c r="I6" s="5">
-        <v>0</v>
-      </c>
-      <c r="J6" s="5">
-        <v>0</v>
-      </c>
-      <c r="K6" s="5">
+      <c r="B6" s="4">
+        <v>0</v>
+      </c>
+      <c r="C6" s="4">
+        <v>0</v>
+      </c>
+      <c r="D6" s="4">
+        <v>0</v>
+      </c>
+      <c r="E6" s="4">
+        <v>0</v>
+      </c>
+      <c r="F6" s="4">
+        <v>1</v>
+      </c>
+      <c r="G6" s="4">
+        <v>0</v>
+      </c>
+      <c r="H6" s="4">
+        <v>0</v>
+      </c>
+      <c r="I6" s="4">
+        <v>0</v>
+      </c>
+      <c r="J6" s="4">
+        <v>0</v>
+      </c>
+      <c r="K6" s="4">
         <v>0</v>
       </c>
     </row>
@@ -720,34 +719,34 @@
       <c r="A7" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="5">
-        <v>0</v>
-      </c>
-      <c r="C7" s="5">
-        <v>0</v>
-      </c>
-      <c r="D7" s="5">
-        <v>0</v>
-      </c>
-      <c r="E7" s="5">
-        <v>0</v>
-      </c>
-      <c r="F7" s="5">
-        <v>0</v>
-      </c>
-      <c r="G7" s="5">
-        <v>1</v>
-      </c>
-      <c r="H7" s="5">
-        <v>0</v>
-      </c>
-      <c r="I7" s="5">
-        <v>0</v>
-      </c>
-      <c r="J7" s="5">
-        <v>0</v>
-      </c>
-      <c r="K7" s="5">
+      <c r="B7" s="4">
+        <v>0</v>
+      </c>
+      <c r="C7" s="4">
+        <v>0</v>
+      </c>
+      <c r="D7" s="4">
+        <v>0</v>
+      </c>
+      <c r="E7" s="4">
+        <v>0</v>
+      </c>
+      <c r="F7" s="4">
+        <v>0</v>
+      </c>
+      <c r="G7" s="4">
+        <v>1</v>
+      </c>
+      <c r="H7" s="4">
+        <v>0</v>
+      </c>
+      <c r="I7" s="4">
+        <v>0</v>
+      </c>
+      <c r="J7" s="4">
+        <v>0</v>
+      </c>
+      <c r="K7" s="4">
         <v>0</v>
       </c>
     </row>
@@ -755,34 +754,34 @@
       <c r="A8" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="5">
-        <v>0</v>
-      </c>
-      <c r="C8" s="5">
-        <v>0</v>
-      </c>
-      <c r="D8" s="5">
-        <v>0</v>
-      </c>
-      <c r="E8" s="5">
-        <v>0</v>
-      </c>
-      <c r="F8" s="5">
-        <v>0</v>
-      </c>
-      <c r="G8" s="5">
-        <v>0</v>
-      </c>
-      <c r="H8" s="5">
-        <v>0</v>
-      </c>
-      <c r="I8" s="5">
-        <v>0</v>
-      </c>
-      <c r="J8" s="5">
-        <v>0</v>
-      </c>
-      <c r="K8" s="5">
+      <c r="B8" s="4">
+        <v>0</v>
+      </c>
+      <c r="C8" s="4">
+        <v>0</v>
+      </c>
+      <c r="D8" s="4">
+        <v>0</v>
+      </c>
+      <c r="E8" s="4">
+        <v>0</v>
+      </c>
+      <c r="F8" s="4">
+        <v>0</v>
+      </c>
+      <c r="G8" s="4">
+        <v>0</v>
+      </c>
+      <c r="H8" s="4">
+        <v>0</v>
+      </c>
+      <c r="I8" s="4">
+        <v>0</v>
+      </c>
+      <c r="J8" s="4">
+        <v>0</v>
+      </c>
+      <c r="K8" s="4">
         <v>0</v>
       </c>
     </row>
@@ -790,34 +789,34 @@
       <c r="A9" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="5">
-        <v>0</v>
-      </c>
-      <c r="C9" s="5">
-        <v>0</v>
-      </c>
-      <c r="D9" s="5">
-        <v>0</v>
-      </c>
-      <c r="E9" s="5">
-        <v>0</v>
-      </c>
-      <c r="F9" s="5">
-        <v>0</v>
-      </c>
-      <c r="G9" s="5">
-        <v>0</v>
-      </c>
-      <c r="H9" s="5">
-        <v>0</v>
-      </c>
-      <c r="I9" s="5">
-        <v>0</v>
-      </c>
-      <c r="J9" s="5">
-        <v>0</v>
-      </c>
-      <c r="K9" s="5">
+      <c r="B9" s="4">
+        <v>0</v>
+      </c>
+      <c r="C9" s="4">
+        <v>0</v>
+      </c>
+      <c r="D9" s="4">
+        <v>0</v>
+      </c>
+      <c r="E9" s="4">
+        <v>0</v>
+      </c>
+      <c r="F9" s="4">
+        <v>0</v>
+      </c>
+      <c r="G9" s="4">
+        <v>0</v>
+      </c>
+      <c r="H9" s="4">
+        <v>0</v>
+      </c>
+      <c r="I9" s="4">
+        <v>0</v>
+      </c>
+      <c r="J9" s="4">
+        <v>0</v>
+      </c>
+      <c r="K9" s="4">
         <v>0</v>
       </c>
     </row>
@@ -825,34 +824,34 @@
       <c r="A10" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="5">
-        <v>0</v>
-      </c>
-      <c r="C10" s="5">
-        <v>0</v>
-      </c>
-      <c r="D10" s="5">
-        <v>0</v>
-      </c>
-      <c r="E10" s="5">
-        <v>0</v>
-      </c>
-      <c r="F10" s="5">
-        <v>0</v>
-      </c>
-      <c r="G10" s="5">
-        <v>0</v>
-      </c>
-      <c r="H10" s="5">
-        <v>0</v>
-      </c>
-      <c r="I10" s="5">
-        <v>0</v>
-      </c>
-      <c r="J10" s="5">
-        <v>0</v>
-      </c>
-      <c r="K10" s="5">
+      <c r="B10" s="4">
+        <v>0</v>
+      </c>
+      <c r="C10" s="4">
+        <v>0</v>
+      </c>
+      <c r="D10" s="4">
+        <v>0</v>
+      </c>
+      <c r="E10" s="4">
+        <v>0</v>
+      </c>
+      <c r="F10" s="4">
+        <v>0</v>
+      </c>
+      <c r="G10" s="4">
+        <v>0</v>
+      </c>
+      <c r="H10" s="4">
+        <v>0</v>
+      </c>
+      <c r="I10" s="4">
+        <v>0</v>
+      </c>
+      <c r="J10" s="4">
+        <v>0</v>
+      </c>
+      <c r="K10" s="4">
         <v>0</v>
       </c>
     </row>
@@ -860,34 +859,34 @@
       <c r="A11" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="5">
-        <v>0</v>
-      </c>
-      <c r="C11" s="5">
-        <v>0</v>
-      </c>
-      <c r="D11" s="5">
-        <v>0</v>
-      </c>
-      <c r="E11" s="5">
-        <v>0</v>
-      </c>
-      <c r="F11" s="5">
-        <v>0</v>
-      </c>
-      <c r="G11" s="5">
-        <v>0</v>
-      </c>
-      <c r="H11" s="5">
-        <v>0</v>
-      </c>
-      <c r="I11" s="5">
-        <v>0</v>
-      </c>
-      <c r="J11" s="5">
-        <v>0</v>
-      </c>
-      <c r="K11" s="5">
+      <c r="B11" s="4">
+        <v>0</v>
+      </c>
+      <c r="C11" s="4">
+        <v>0</v>
+      </c>
+      <c r="D11" s="4">
+        <v>0</v>
+      </c>
+      <c r="E11" s="4">
+        <v>0</v>
+      </c>
+      <c r="F11" s="4">
+        <v>0</v>
+      </c>
+      <c r="G11" s="4">
+        <v>0</v>
+      </c>
+      <c r="H11" s="4">
+        <v>0</v>
+      </c>
+      <c r="I11" s="4">
+        <v>0</v>
+      </c>
+      <c r="J11" s="4">
+        <v>0</v>
+      </c>
+      <c r="K11" s="4">
         <v>0</v>
       </c>
     </row>

</xml_diff>